<commit_message>
validade externa - c2 - atualizacao da tabela
</commit_message>
<xml_diff>
--- a/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
+++ b/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fed8d7a7efb8cd6/Trampos/Cebrap/Afro/Projetos/Territorio Negro/analysis/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fed8d7a7efb8cd6/Trampos/Cebrap/Afro/Projetos/Territorio Negro/analysis/territorios_negros/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95377381-C4A5-44E8-97EE-0C42FA7E5673}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{914DFB8F-F030-4E1F-A71F-EE37ED9CC392}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{FB758A09-3C3B-4901-8572-23A69892CF1B}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="35">
   <si>
     <t>RM</t>
   </si>
@@ -146,12 +146,18 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Var. rel. (%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -181,10 +187,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -521,20 +533,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2B67E7F-2C6F-44EC-9EDA-D675DEA86371}">
-  <dimension ref="B2:J11"/>
+  <dimension ref="B2:K11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" customWidth="1"/>
-    <col min="7" max="7" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -551,195 +564,276 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
         <v>0.31</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>0.33</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>0.28999999999999998</v>
       </c>
-      <c r="G3" t="s">
+      <c r="F3" s="2">
+        <f>C3-D3</f>
+        <v>-2.0000000000000018E-2</v>
+      </c>
+      <c r="G3" s="4">
+        <f>F3/D3*100</f>
+        <v>-6.0606060606060659</v>
+      </c>
+      <c r="H3" t="s">
         <v>26</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>14</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>5</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="3">
         <v>0.22</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>0.32</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="3">
         <v>0.27</v>
       </c>
-      <c r="G4" t="s">
+      <c r="F4" s="2">
+        <f t="shared" ref="F4:F11" si="0">C4-D4</f>
+        <v>-0.1</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" ref="G4:G11" si="1">F4/D4*100</f>
+        <v>-31.25</v>
+      </c>
+      <c r="H4" t="s">
         <v>19</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>5</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="3">
         <v>0.22</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>0.21</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="3">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F5" s="2">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="1"/>
+        <v>4.7619047619047663</v>
+      </c>
+      <c r="H5" t="s">
         <v>19</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>5</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="3">
         <v>0.22</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>0.22</v>
       </c>
-      <c r="G6" t="s">
+      <c r="E6" s="3"/>
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
         <v>19</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="3">
         <v>0.26</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="2">
         <v>0.28999999999999998</v>
       </c>
-      <c r="G7" t="s">
+      <c r="E7" s="3"/>
+      <c r="F7" s="2">
+        <f t="shared" si="0"/>
+        <v>-2.9999999999999971E-2</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="1"/>
+        <v>-10.344827586206886</v>
+      </c>
+      <c r="H7" t="s">
         <v>19</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="3">
         <v>0.27</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>0.3</v>
       </c>
-      <c r="G8" t="s">
+      <c r="E8" s="3"/>
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>-2.9999999999999971E-2</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="1"/>
+        <v>-9.9999999999999911</v>
+      </c>
+      <c r="H8" t="s">
         <v>19</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>23</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="3">
         <v>0.32</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="2">
         <v>0.33</v>
       </c>
-      <c r="G9" t="s">
+      <c r="E9" s="3"/>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>-1.0000000000000009E-2</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" si="1"/>
+        <v>-3.0303030303030329</v>
+      </c>
+      <c r="H9" t="s">
         <v>19</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="2">
         <v>0.3</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="2">
         <v>0.3</v>
       </c>
-      <c r="G10" t="s">
+      <c r="E10" s="3"/>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
         <v>19</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="3">
         <v>0.34</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="2">
         <v>0.34</v>
       </c>
-      <c r="G11" t="s">
+      <c r="E11" s="3"/>
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
         <v>19</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>17</v>
       </c>
     </row>
@@ -978,20 +1072,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E28EE20A-9A43-46EF-9D96-67853D17F860}">
-  <dimension ref="B2:J15"/>
+  <dimension ref="B2:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1007,20 +1101,20 @@
       <c r="F2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>28</v>
       </c>
@@ -1030,14 +1124,22 @@
       <c r="D3">
         <v>0.28999999999999998</v>
       </c>
-      <c r="G3" t="s">
+      <c r="F3" s="2">
+        <f>C3-D3</f>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G3" s="4">
+        <f>F3/D3*100</f>
+        <v>3.4482758620689689</v>
+      </c>
+      <c r="H3" t="s">
         <v>32</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>20</v>
       </c>
@@ -1047,14 +1149,22 @@
       <c r="D4">
         <v>0.43</v>
       </c>
-      <c r="G4" t="s">
+      <c r="F4" s="2">
+        <f t="shared" ref="F4:F11" si="0">C4-D4</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" ref="G4:G11" si="1">F4/D4*100</f>
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>32</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>8</v>
       </c>
@@ -1064,14 +1174,22 @@
       <c r="D5">
         <v>0.39</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F5" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
         <v>32</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1081,14 +1199,22 @@
       <c r="D6">
         <v>0.28000000000000003</v>
       </c>
-      <c r="G6" t="s">
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
+        <v>9.9999999999999534E-3</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285547</v>
+      </c>
+      <c r="H6" t="s">
         <v>32</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>21</v>
       </c>
@@ -1098,14 +1224,22 @@
       <c r="D7">
         <v>0.48</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F7" s="2">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="1"/>
+        <v>2.0833333333333353</v>
+      </c>
+      <c r="H7" t="s">
         <v>32</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>22</v>
       </c>
@@ -1115,14 +1249,22 @@
       <c r="D8">
         <v>0.54</v>
       </c>
-      <c r="G8" t="s">
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
         <v>32</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>29</v>
       </c>
@@ -1132,14 +1274,20 @@
       <c r="D9">
         <v>0.45</v>
       </c>
-      <c r="G9" t="s">
+      <c r="F9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
         <v>32</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -1149,14 +1297,22 @@
       <c r="D10">
         <v>0.49</v>
       </c>
-      <c r="G10" t="s">
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
         <v>32</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>6</v>
       </c>
@@ -1169,20 +1325,28 @@
       <c r="E11">
         <v>1.05</v>
       </c>
-      <c r="G11" t="s">
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000018E-2</v>
+      </c>
+      <c r="G11" s="4">
+        <f t="shared" si="1"/>
+        <v>3.1250000000000027</v>
+      </c>
+      <c r="H11" t="s">
         <v>32</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>27</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>15</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>31</v>
       </c>
@@ -1192,14 +1356,22 @@
       <c r="D12">
         <v>0.63</v>
       </c>
-      <c r="G12" t="s">
+      <c r="F12" s="2">
+        <f>C12-D12</f>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G12" s="4">
+        <f>F12/D12*100</f>
+        <v>1.5873015873015885</v>
+      </c>
+      <c r="H12" t="s">
         <v>32</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>23</v>
       </c>
@@ -1209,14 +1381,22 @@
       <c r="D13">
         <v>0.71</v>
       </c>
-      <c r="G13" t="s">
+      <c r="F13" s="2">
+        <f t="shared" ref="F13:F15" si="2">C13-D13</f>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G13" s="4">
+        <f t="shared" ref="G13:G15" si="3">F13/D13*100</f>
+        <v>1.4084507042253533</v>
+      </c>
+      <c r="H13" t="s">
         <v>32</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>24</v>
       </c>
@@ -1226,14 +1406,22 @@
       <c r="D14">
         <v>0.77</v>
       </c>
-      <c r="G14" t="s">
+      <c r="F14" s="2">
+        <f t="shared" si="2"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G14" s="4">
+        <f t="shared" si="3"/>
+        <v>1.2987012987012998</v>
+      </c>
+      <c r="H14" t="s">
         <v>32</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>25</v>
       </c>
@@ -1243,10 +1431,18 @@
       <c r="D15">
         <v>0.84</v>
       </c>
-      <c r="G15" t="s">
+      <c r="F15" s="2">
+        <f t="shared" si="2"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G15" s="4">
+        <f t="shared" si="3"/>
+        <v>1.1904761904761916</v>
+      </c>
+      <c r="H15" t="s">
         <v>32</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>